<commit_message>
Fix open access PDF links and update site
</commit_message>
<xml_diff>
--- a/data/publications.xlsx
+++ b/data/publications.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\E-library\Vowan_Database\Valentine_Site_Clean\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89062621-2D58-4F5F-B517-B89D68D010EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCCE0DA2-9A38-48F7-A3A4-8B482A338988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4192" uniqueCount="2845">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4216" uniqueCount="2869">
   <si>
     <t>slug</t>
   </si>
@@ -10183,6 +10183,78 @@
   </si>
   <si>
     <t>bedproject</t>
+  </si>
+  <si>
+    <t>assets/papers/articles/2024/odiong-et-al-2024-data-accessibility-research-attitude.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/articles/2024/ekpenyong-et-al-2024-principals-managerial-behaviour-school-climate.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/articles/2023/idika-owan-agama-2023-nominal-scale-measurement.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/chapters/2022/owan-asuquo-2022-publish-or-perish-nigerian-experience.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/chapters/2022/odigwe-owan-2022-collaborative-research-wealth-creation.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/articles/2022/owan-agurokpon-owan-2022-primary-schools-libraries-texts-core-subjects.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/articles/2021/owan-et-al-2021-online-platforms-research-dissemination.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/articles/2021/owan-et-al-2021-library-resources-lesson-preparation.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/articles/2021/owan-et-al-2021-gender-age-preparedness-internet-tools-research-sharing.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/articles/2021/aslam-sonkar-owan-2021-teaching-learning-covid19-lockdown-lis-india.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/chapters/2020/bassey-owan-2020-higher-ordered-test-items-pandemics.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/chapters/2020/owan-2020-computer-administered-testing-sars-related-outbreaks.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/articles/2019/robert-owan-2019-teachers-effectiveness-learning-outcomes-mathematics-economics.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/articles/2019/bassey-owan-eze-2019-nexus-students-teachers-school-system-effectiveness-instrument.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/articles/2019/arop-owan-agunwa-2019-teaching-personnel-management-attitude-to-work-calabar.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/articles/2019/offem-arop-owan-2019-management-of-discipline-academic-performance-cross-river.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/articles/2019/arop-owan-ibor-2019-school-quality-indicators-teachers-job-performance-cross-river.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/articles/2019/egbula-arop-owan-2019-practicum-exercise-attitudes-pre-service-educational-administrators.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/articles/2019/arop-agunwa-owan-2019-tertiary-students-social-media-management-attitudes-academic-performance.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/articles/2019/arop-owan-madukwe-2019-human-resource-management-teachers-job-performance-akamkpa.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/articles/2019/owan-arop-agunwa-2019-path-analysis-innovative-management-practices-school-system-effectiveness.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/articles/2019/owan-duruamaku-dim-eneje-2019-mode-test-administration-birth-variables-mathematics-achievement.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/projects/2018-bachelor-project.pdf</t>
+  </si>
+  <si>
+    <t>assets/papers/projects/2012-nce-project.pdf</t>
   </si>
 </sst>
 </file>
@@ -12099,6 +12171,9 @@
       <c r="R18" t="s">
         <v>335</v>
       </c>
+      <c r="S18" t="s">
+        <v>2845</v>
+      </c>
       <c r="T18" t="s">
         <v>49</v>
       </c>
@@ -12170,6 +12245,9 @@
       <c r="R19" t="s">
         <v>350</v>
       </c>
+      <c r="S19" t="s">
+        <v>2846</v>
+      </c>
       <c r="T19" t="s">
         <v>49</v>
       </c>
@@ -14097,6 +14175,9 @@
       <c r="R39" t="s">
         <v>726</v>
       </c>
+      <c r="S39" t="s">
+        <v>2847</v>
+      </c>
       <c r="T39" t="s">
         <v>49</v>
       </c>
@@ -15926,6 +16007,9 @@
       <c r="O58" t="s">
         <v>1083</v>
       </c>
+      <c r="S58" t="s">
+        <v>2848</v>
+      </c>
       <c r="T58" t="s">
         <v>49</v>
       </c>
@@ -15988,6 +16072,9 @@
       <c r="O59" t="s">
         <v>1095</v>
       </c>
+      <c r="S59" t="s">
+        <v>2849</v>
+      </c>
       <c r="T59" t="s">
         <v>49</v>
       </c>
@@ -17918,6 +18005,9 @@
       <c r="R79" t="s">
         <v>1461</v>
       </c>
+      <c r="S79" t="s">
+        <v>2850</v>
+      </c>
       <c r="T79" t="s">
         <v>49</v>
       </c>
@@ -18114,6 +18204,9 @@
       <c r="R81" t="s">
         <v>1497</v>
       </c>
+      <c r="S81" t="s">
+        <v>2851</v>
+      </c>
       <c r="T81" t="s">
         <v>49</v>
       </c>
@@ -18506,6 +18599,9 @@
       <c r="R85" t="s">
         <v>1573</v>
       </c>
+      <c r="S85" t="s">
+        <v>2852</v>
+      </c>
       <c r="T85" t="s">
         <v>49</v>
       </c>
@@ -18601,6 +18697,9 @@
       <c r="R86" t="s">
         <v>1590</v>
       </c>
+      <c r="S86" t="s">
+        <v>2853</v>
+      </c>
       <c r="T86" t="s">
         <v>49</v>
       </c>
@@ -18892,6 +18991,9 @@
       <c r="R89" t="s">
         <v>1645</v>
       </c>
+      <c r="S89" t="s">
+        <v>2854</v>
+      </c>
       <c r="T89" t="s">
         <v>49</v>
       </c>
@@ -19382,6 +19484,9 @@
       <c r="O94" t="s">
         <v>1735</v>
       </c>
+      <c r="S94" t="s">
+        <v>2856</v>
+      </c>
       <c r="T94" t="s">
         <v>49</v>
       </c>
@@ -19468,6 +19573,9 @@
       <c r="O95" t="s">
         <v>1748</v>
       </c>
+      <c r="S95" t="s">
+        <v>2855</v>
+      </c>
       <c r="T95" t="s">
         <v>49</v>
       </c>
@@ -22414,6 +22522,9 @@
       <c r="R125" t="s">
         <v>2296</v>
       </c>
+      <c r="S125" t="s">
+        <v>2857</v>
+      </c>
       <c r="T125" t="s">
         <v>49</v>
       </c>
@@ -22708,6 +22819,9 @@
       <c r="R128" t="s">
         <v>2351</v>
       </c>
+      <c r="S128" t="s">
+        <v>2858</v>
+      </c>
       <c r="T128" t="s">
         <v>49</v>
       </c>
@@ -22803,6 +22917,9 @@
       <c r="R129" t="s">
         <v>2367</v>
       </c>
+      <c r="S129" t="s">
+        <v>2859</v>
+      </c>
       <c r="T129" t="s">
         <v>49</v>
       </c>
@@ -22999,6 +23116,9 @@
       <c r="R131" t="s">
         <v>2403</v>
       </c>
+      <c r="S131" t="s">
+        <v>2862</v>
+      </c>
       <c r="T131" t="s">
         <v>49</v>
       </c>
@@ -23094,6 +23214,9 @@
       <c r="R132" t="s">
         <v>2419</v>
       </c>
+      <c r="S132" t="s">
+        <v>2861</v>
+      </c>
       <c r="T132" t="s">
         <v>49</v>
       </c>
@@ -23189,6 +23312,9 @@
       <c r="R133" t="s">
         <v>2436</v>
       </c>
+      <c r="S133" t="s">
+        <v>2860</v>
+      </c>
       <c r="T133" t="s">
         <v>49</v>
       </c>
@@ -23486,6 +23612,9 @@
       <c r="R136" t="s">
         <v>2490</v>
       </c>
+      <c r="S136" t="s">
+        <v>2864</v>
+      </c>
       <c r="T136" t="s">
         <v>49</v>
       </c>
@@ -23581,6 +23710,9 @@
       <c r="R137" t="s">
         <v>2506</v>
       </c>
+      <c r="S137" t="s">
+        <v>2863</v>
+      </c>
       <c r="T137" t="s">
         <v>49</v>
       </c>
@@ -23676,6 +23808,9 @@
       <c r="R138" t="s">
         <v>2521</v>
       </c>
+      <c r="S138" t="s">
+        <v>2865</v>
+      </c>
       <c r="T138" t="s">
         <v>49</v>
       </c>
@@ -23869,6 +24004,9 @@
       <c r="R140" t="s">
         <v>2556</v>
       </c>
+      <c r="S140" t="s">
+        <v>2866</v>
+      </c>
       <c r="T140" t="s">
         <v>49</v>
       </c>
@@ -24163,6 +24301,9 @@
       <c r="Q143" t="s">
         <v>2612</v>
       </c>
+      <c r="S143" t="s">
+        <v>2867</v>
+      </c>
       <c r="T143" t="s">
         <v>49</v>
       </c>
@@ -25424,6 +25565,9 @@
       </c>
       <c r="Q156" t="s">
         <v>2834</v>
+      </c>
+      <c r="S156" t="s">
+        <v>2868</v>
       </c>
       <c r="T156" t="s">
         <v>49</v>

</xml_diff>

<commit_message>
Automate homepage recent publications
</commit_message>
<xml_diff>
--- a/data/publications.xlsx
+++ b/data/publications.xlsx
@@ -9580,13 +9580,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -21770,7 +21769,7 @@
       <c r="T162" t="s">
         <v>52</v>
       </c>
-      <c r="Z162" s="3" t="s">
+      <c r="Z162" t="s">
         <v>2584</v>
       </c>
       <c r="AD162" t="s">
@@ -21802,7 +21801,7 @@
       <c r="C163" t="s">
         <v>42</v>
       </c>
-      <c r="D163" s="4" t="s">
+      <c r="D163" s="3" t="s">
         <v>2592</v>
       </c>
       <c r="E163">
@@ -21861,10 +21860,10 @@
       </c>
     </row>
     <row r="164" spans="1:35">
-      <c r="A164" s="4" t="s">
+      <c r="A164" s="3" t="s">
         <v>2606</v>
       </c>
-      <c r="B164" s="3" t="s">
+      <c r="B164" t="s">
         <v>2607</v>
       </c>
       <c r="C164" t="s">

</xml_diff>

<commit_message>
retouch of the recent publications
</commit_message>
<xml_diff>
--- a/data/publications.xlsx
+++ b/data/publications.xlsx
@@ -698,7 +698,11 @@
           <t>assets/papers/articles/2027/ogabor-et-al-2027-aerobic-exercise-on-biopsychological-function-msj-brazil.pdf</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
@@ -872,7 +876,7 @@
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr"/>
@@ -1019,7 +1023,7 @@
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr"/>
@@ -1153,7 +1157,7 @@
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr"/>
@@ -1287,7 +1291,7 @@
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr"/>
@@ -1563,7 +1567,7 @@
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr"/>
@@ -1708,7 +1712,7 @@
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr"/>
@@ -2123,7 +2127,7 @@
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD12" t="inlineStr"/>
@@ -2268,7 +2272,7 @@
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD13" t="inlineStr"/>
@@ -2650,7 +2654,7 @@
       </c>
       <c r="AC16" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD16" t="inlineStr"/>
@@ -2795,7 +2799,7 @@
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD17" t="inlineStr"/>
@@ -2940,7 +2944,7 @@
       </c>
       <c r="AC18" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD18" t="inlineStr"/>
@@ -3085,7 +3089,7 @@
       </c>
       <c r="AC19" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD19" t="inlineStr"/>
@@ -3230,7 +3234,7 @@
       </c>
       <c r="AC20" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD20" t="inlineStr"/>
@@ -3375,7 +3379,7 @@
       </c>
       <c r="AC21" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD21" t="inlineStr"/>
@@ -3925,7 +3929,7 @@
       </c>
       <c r="AC25" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD25" t="inlineStr"/>
@@ -4071,7 +4075,7 @@
       </c>
       <c r="AC26" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD26" t="inlineStr"/>
@@ -4481,7 +4485,7 @@
       </c>
       <c r="AC29" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD29" t="inlineStr"/>
@@ -4628,7 +4632,7 @@
       </c>
       <c r="AC30" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD30" t="inlineStr"/>
@@ -4773,7 +4777,7 @@
       </c>
       <c r="AC31" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD31" t="inlineStr"/>
@@ -4918,7 +4922,7 @@
       </c>
       <c r="AC32" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD32" t="inlineStr"/>
@@ -5063,7 +5067,7 @@
       </c>
       <c r="AC33" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD33" t="inlineStr"/>
@@ -5202,7 +5206,7 @@
       </c>
       <c r="AC34" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD34" t="inlineStr"/>
@@ -5352,7 +5356,7 @@
       </c>
       <c r="AC35" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD35" t="inlineStr"/>
@@ -5497,7 +5501,7 @@
       </c>
       <c r="AC36" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD36" t="inlineStr"/>
@@ -5635,7 +5639,7 @@
       </c>
       <c r="AC37" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD37" t="inlineStr"/>
@@ -5779,7 +5783,7 @@
       </c>
       <c r="AC38" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD38" t="inlineStr"/>
@@ -5924,7 +5928,7 @@
       </c>
       <c r="AC39" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD39" t="inlineStr"/>
@@ -6069,7 +6073,7 @@
       </c>
       <c r="AC40" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD40" t="inlineStr"/>
@@ -6214,7 +6218,7 @@
       </c>
       <c r="AC41" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD41" t="inlineStr"/>
@@ -6353,7 +6357,7 @@
       </c>
       <c r="AC42" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD42" t="inlineStr"/>
@@ -6492,7 +6496,7 @@
       </c>
       <c r="AC43" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD43" t="inlineStr"/>
@@ -6631,7 +6635,7 @@
       </c>
       <c r="AC44" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD44" t="inlineStr"/>
@@ -6770,7 +6774,7 @@
       </c>
       <c r="AC45" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD45" t="inlineStr"/>
@@ -6915,7 +6919,7 @@
       </c>
       <c r="AC46" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD46" t="inlineStr"/>
@@ -7060,7 +7064,7 @@
       </c>
       <c r="AC47" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD47" t="inlineStr"/>
@@ -7339,7 +7343,7 @@
       </c>
       <c r="AC49" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD49" t="inlineStr"/>
@@ -7484,7 +7488,7 @@
       </c>
       <c r="AC50" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD50" t="inlineStr"/>
@@ -7758,7 +7762,7 @@
       </c>
       <c r="AC52" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD52" t="inlineStr"/>
@@ -7908,7 +7912,7 @@
       </c>
       <c r="AC53" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD53" t="inlineStr"/>
@@ -8053,7 +8057,7 @@
       </c>
       <c r="AC54" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD54" t="inlineStr"/>
@@ -8198,7 +8202,7 @@
       </c>
       <c r="AC55" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD55" t="inlineStr"/>
@@ -8343,7 +8347,7 @@
       </c>
       <c r="AC56" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD56" t="inlineStr"/>
@@ -8488,7 +8492,7 @@
       </c>
       <c r="AC57" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD57" t="inlineStr"/>
@@ -8633,7 +8637,7 @@
       </c>
       <c r="AC58" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD58" t="inlineStr"/>
@@ -8775,7 +8779,7 @@
       </c>
       <c r="AC59" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD59" t="inlineStr"/>
@@ -9055,7 +9059,7 @@
       </c>
       <c r="AC61" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD61" t="inlineStr"/>
@@ -9197,7 +9201,7 @@
       </c>
       <c r="AC62" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD62" t="inlineStr"/>
@@ -9342,7 +9346,7 @@
       </c>
       <c r="AC63" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD63" t="inlineStr"/>
@@ -9487,7 +9491,7 @@
       </c>
       <c r="AC64" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD64" t="inlineStr"/>
@@ -9632,7 +9636,7 @@
       </c>
       <c r="AC65" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD65" t="inlineStr"/>
@@ -9782,7 +9786,7 @@
       </c>
       <c r="AC66" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD66" t="inlineStr"/>
@@ -10170,7 +10174,7 @@
       </c>
       <c r="AC69" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD69" t="inlineStr"/>
@@ -10312,7 +10316,7 @@
       </c>
       <c r="AC70" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD70" t="inlineStr"/>
@@ -10457,7 +10461,7 @@
       </c>
       <c r="AC71" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD71" t="inlineStr"/>
@@ -10602,7 +10606,7 @@
       </c>
       <c r="AC72" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD72" t="inlineStr"/>
@@ -10747,7 +10751,7 @@
       </c>
       <c r="AC73" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD73" t="inlineStr"/>
@@ -10888,7 +10892,7 @@
       </c>
       <c r="AC74" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD74" t="inlineStr"/>
@@ -11033,7 +11037,7 @@
       </c>
       <c r="AC75" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD75" t="inlineStr"/>
@@ -11178,7 +11182,7 @@
       </c>
       <c r="AC76" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD76" t="inlineStr"/>
@@ -11320,7 +11324,7 @@
       </c>
       <c r="AC77" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD77" t="inlineStr"/>
@@ -11459,7 +11463,7 @@
       </c>
       <c r="AC78" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD78" t="inlineStr"/>
@@ -11598,7 +11602,7 @@
       </c>
       <c r="AC79" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD79" t="inlineStr"/>
@@ -11737,7 +11741,7 @@
       </c>
       <c r="AC80" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD80" t="inlineStr"/>
@@ -11876,7 +11880,7 @@
       </c>
       <c r="AC81" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD81" t="inlineStr"/>
@@ -12026,7 +12030,7 @@
       </c>
       <c r="AC82" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD82" t="inlineStr"/>
@@ -12171,7 +12175,7 @@
       </c>
       <c r="AC83" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD83" t="inlineStr"/>
@@ -12316,7 +12320,7 @@
       </c>
       <c r="AC84" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD84" t="inlineStr"/>
@@ -12461,7 +12465,7 @@
       </c>
       <c r="AC85" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD85" t="inlineStr"/>
@@ -12606,7 +12610,7 @@
       </c>
       <c r="AC86" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD86" t="inlineStr"/>
@@ -12748,7 +12752,7 @@
       </c>
       <c r="AC87" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD87" t="inlineStr"/>
@@ -13024,7 +13028,7 @@
       </c>
       <c r="AC89" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD89" t="inlineStr"/>
@@ -13300,7 +13304,7 @@
       </c>
       <c r="AC91" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD91" t="inlineStr"/>
@@ -13445,7 +13449,7 @@
       </c>
       <c r="AC92" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD92" t="inlineStr"/>
@@ -13590,7 +13594,7 @@
       </c>
       <c r="AC93" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD93" t="inlineStr"/>
@@ -13994,7 +13998,7 @@
       </c>
       <c r="AC96" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD96" t="inlineStr"/>
@@ -14139,7 +14143,7 @@
       </c>
       <c r="AC97" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD97" t="inlineStr"/>
@@ -14415,7 +14419,7 @@
       </c>
       <c r="AC99" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD99" t="inlineStr"/>
@@ -14560,7 +14564,7 @@
       </c>
       <c r="AC100" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD100" t="inlineStr"/>
@@ -14705,7 +14709,7 @@
       </c>
       <c r="AC101" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD101" t="inlineStr"/>
@@ -14850,7 +14854,7 @@
       </c>
       <c r="AC102" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD102" t="inlineStr"/>
@@ -15240,7 +15244,7 @@
       </c>
       <c r="AC105" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD105" t="inlineStr"/>
@@ -15385,7 +15389,7 @@
       </c>
       <c r="AC106" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD106" t="inlineStr"/>
@@ -15530,7 +15534,7 @@
       </c>
       <c r="AC107" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD107" t="inlineStr"/>
@@ -15675,7 +15679,7 @@
       </c>
       <c r="AC108" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD108" t="inlineStr"/>
@@ -15819,7 +15823,7 @@
       </c>
       <c r="AC109" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD109" t="inlineStr"/>
@@ -15964,7 +15968,7 @@
       </c>
       <c r="AC110" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD110" t="inlineStr"/>
@@ -16109,7 +16113,7 @@
       </c>
       <c r="AC111" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD111" t="inlineStr"/>
@@ -16254,7 +16258,7 @@
       </c>
       <c r="AC112" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD112" t="inlineStr"/>
@@ -16399,7 +16403,7 @@
       </c>
       <c r="AC113" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD113" t="inlineStr"/>
@@ -16544,7 +16548,7 @@
       </c>
       <c r="AC114" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD114" t="inlineStr"/>
@@ -16689,7 +16693,7 @@
       </c>
       <c r="AC115" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD115" t="inlineStr"/>
@@ -16834,7 +16838,7 @@
       </c>
       <c r="AC116" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD116" t="inlineStr"/>
@@ -16979,7 +16983,7 @@
       </c>
       <c r="AC117" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD117" t="inlineStr"/>
@@ -17124,7 +17128,7 @@
       </c>
       <c r="AC118" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD118" t="inlineStr"/>
@@ -17269,7 +17273,7 @@
       </c>
       <c r="AC119" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD119" t="inlineStr"/>
@@ -17414,7 +17418,7 @@
       </c>
       <c r="AC120" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD120" t="inlineStr"/>
@@ -17559,7 +17563,7 @@
       </c>
       <c r="AC121" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD121" t="inlineStr"/>
@@ -17704,7 +17708,7 @@
       </c>
       <c r="AC122" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD122" t="inlineStr"/>
@@ -17982,7 +17986,7 @@
       </c>
       <c r="AC124" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD124" t="inlineStr"/>
@@ -18666,7 +18670,7 @@
       </c>
       <c r="AC129" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD129" t="inlineStr"/>
@@ -18810,7 +18814,7 @@
       </c>
       <c r="AC130" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD130" t="inlineStr"/>
@@ -19225,7 +19229,7 @@
       </c>
       <c r="AC133" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD133" t="inlineStr"/>
@@ -19504,7 +19508,7 @@
       </c>
       <c r="AC135" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD135" t="inlineStr"/>
@@ -19649,7 +19653,7 @@
       </c>
       <c r="AC136" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD136" t="inlineStr"/>
@@ -20062,7 +20066,7 @@
       </c>
       <c r="AC139" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD139" t="inlineStr"/>
@@ -20609,7 +20613,7 @@
       </c>
       <c r="AC143" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD143" t="inlineStr"/>
@@ -21695,7 +21699,7 @@
       </c>
       <c r="AC151" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD151" t="inlineStr"/>
@@ -21838,7 +21842,7 @@
       </c>
       <c r="AC152" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD152" t="inlineStr"/>
@@ -22118,7 +22122,7 @@
       </c>
       <c r="AC154" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD154" t="inlineStr"/>
@@ -22263,7 +22267,7 @@
       </c>
       <c r="AC155" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD155" t="inlineStr"/>
@@ -22678,7 +22682,7 @@
       </c>
       <c r="AC158" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD158" t="inlineStr"/>
@@ -23093,7 +23097,7 @@
       </c>
       <c r="AC161" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD161" t="inlineStr"/>
@@ -23373,7 +23377,7 @@
       </c>
       <c r="AC163" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD163" t="inlineStr"/>
@@ -23646,7 +23650,7 @@
       </c>
       <c r="AC165" t="inlineStr">
         <is>
-          <t>2026-08-15 06:53:05</t>
+          <t>2026-08-15 07:08:06</t>
         </is>
       </c>
       <c r="AD165" t="inlineStr"/>

</xml_diff>

<commit_message>
Fix publication links and update database
</commit_message>
<xml_diff>
--- a/data/publications.xlsx
+++ b/data/publications.xlsx
@@ -621,7 +621,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2027-ogabor-et-al-aerobic-exercise-on-biopsychological-function-msj-brazil.html</t>
+          <t>2027-ogabor-et-al-aerobic-exercise-on-biopsychological-function-msj-brazil</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -876,7 +876,7 @@
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr"/>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr"/>
@@ -1157,7 +1157,7 @@
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr"/>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr"/>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr"/>
@@ -1712,7 +1712,7 @@
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr"/>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD12" t="inlineStr"/>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD13" t="inlineStr"/>
@@ -2654,7 +2654,7 @@
       </c>
       <c r="AC16" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD16" t="inlineStr"/>
@@ -2799,7 +2799,7 @@
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD17" t="inlineStr"/>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="AC18" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD18" t="inlineStr"/>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="AC19" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD19" t="inlineStr"/>
@@ -3234,7 +3234,7 @@
       </c>
       <c r="AC20" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD20" t="inlineStr"/>
@@ -3379,7 +3379,7 @@
       </c>
       <c r="AC21" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD21" t="inlineStr"/>
@@ -3929,7 +3929,7 @@
       </c>
       <c r="AC25" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD25" t="inlineStr"/>
@@ -4075,7 +4075,7 @@
       </c>
       <c r="AC26" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD26" t="inlineStr"/>
@@ -4485,7 +4485,7 @@
       </c>
       <c r="AC29" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD29" t="inlineStr"/>
@@ -4632,7 +4632,7 @@
       </c>
       <c r="AC30" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD30" t="inlineStr"/>
@@ -4777,7 +4777,7 @@
       </c>
       <c r="AC31" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD31" t="inlineStr"/>
@@ -4922,7 +4922,7 @@
       </c>
       <c r="AC32" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD32" t="inlineStr"/>
@@ -5067,7 +5067,7 @@
       </c>
       <c r="AC33" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD33" t="inlineStr"/>
@@ -5206,7 +5206,7 @@
       </c>
       <c r="AC34" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD34" t="inlineStr"/>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="AC35" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD35" t="inlineStr"/>
@@ -5501,7 +5501,7 @@
       </c>
       <c r="AC36" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD36" t="inlineStr"/>
@@ -5639,7 +5639,7 @@
       </c>
       <c r="AC37" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD37" t="inlineStr"/>
@@ -5783,7 +5783,7 @@
       </c>
       <c r="AC38" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD38" t="inlineStr"/>
@@ -5928,7 +5928,7 @@
       </c>
       <c r="AC39" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD39" t="inlineStr"/>
@@ -6073,7 +6073,7 @@
       </c>
       <c r="AC40" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD40" t="inlineStr"/>
@@ -6218,7 +6218,7 @@
       </c>
       <c r="AC41" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD41" t="inlineStr"/>
@@ -6357,7 +6357,7 @@
       </c>
       <c r="AC42" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD42" t="inlineStr"/>
@@ -6496,7 +6496,7 @@
       </c>
       <c r="AC43" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD43" t="inlineStr"/>
@@ -6635,7 +6635,7 @@
       </c>
       <c r="AC44" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD44" t="inlineStr"/>
@@ -6774,7 +6774,7 @@
       </c>
       <c r="AC45" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD45" t="inlineStr"/>
@@ -6919,7 +6919,7 @@
       </c>
       <c r="AC46" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD46" t="inlineStr"/>
@@ -7064,7 +7064,7 @@
       </c>
       <c r="AC47" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD47" t="inlineStr"/>
@@ -7343,7 +7343,7 @@
       </c>
       <c r="AC49" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD49" t="inlineStr"/>
@@ -7488,7 +7488,7 @@
       </c>
       <c r="AC50" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD50" t="inlineStr"/>
@@ -7762,7 +7762,7 @@
       </c>
       <c r="AC52" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD52" t="inlineStr"/>
@@ -7912,7 +7912,7 @@
       </c>
       <c r="AC53" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD53" t="inlineStr"/>
@@ -8057,7 +8057,7 @@
       </c>
       <c r="AC54" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD54" t="inlineStr"/>
@@ -8202,7 +8202,7 @@
       </c>
       <c r="AC55" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD55" t="inlineStr"/>
@@ -8347,7 +8347,7 @@
       </c>
       <c r="AC56" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD56" t="inlineStr"/>
@@ -8492,7 +8492,7 @@
       </c>
       <c r="AC57" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD57" t="inlineStr"/>
@@ -8637,7 +8637,7 @@
       </c>
       <c r="AC58" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD58" t="inlineStr"/>
@@ -8779,7 +8779,7 @@
       </c>
       <c r="AC59" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD59" t="inlineStr"/>
@@ -9059,7 +9059,7 @@
       </c>
       <c r="AC61" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD61" t="inlineStr"/>
@@ -9201,7 +9201,7 @@
       </c>
       <c r="AC62" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD62" t="inlineStr"/>
@@ -9346,7 +9346,7 @@
       </c>
       <c r="AC63" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD63" t="inlineStr"/>
@@ -9491,7 +9491,7 @@
       </c>
       <c r="AC64" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD64" t="inlineStr"/>
@@ -9636,7 +9636,7 @@
       </c>
       <c r="AC65" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD65" t="inlineStr"/>
@@ -9786,7 +9786,7 @@
       </c>
       <c r="AC66" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD66" t="inlineStr"/>
@@ -10174,7 +10174,7 @@
       </c>
       <c r="AC69" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD69" t="inlineStr"/>
@@ -10316,7 +10316,7 @@
       </c>
       <c r="AC70" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD70" t="inlineStr"/>
@@ -10461,7 +10461,7 @@
       </c>
       <c r="AC71" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD71" t="inlineStr"/>
@@ -10606,7 +10606,7 @@
       </c>
       <c r="AC72" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD72" t="inlineStr"/>
@@ -10751,7 +10751,7 @@
       </c>
       <c r="AC73" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD73" t="inlineStr"/>
@@ -10892,7 +10892,7 @@
       </c>
       <c r="AC74" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD74" t="inlineStr"/>
@@ -11037,7 +11037,7 @@
       </c>
       <c r="AC75" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD75" t="inlineStr"/>
@@ -11182,7 +11182,7 @@
       </c>
       <c r="AC76" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD76" t="inlineStr"/>
@@ -11324,7 +11324,7 @@
       </c>
       <c r="AC77" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD77" t="inlineStr"/>
@@ -11463,7 +11463,7 @@
       </c>
       <c r="AC78" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD78" t="inlineStr"/>
@@ -11602,7 +11602,7 @@
       </c>
       <c r="AC79" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD79" t="inlineStr"/>
@@ -11741,7 +11741,7 @@
       </c>
       <c r="AC80" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD80" t="inlineStr"/>
@@ -11880,7 +11880,7 @@
       </c>
       <c r="AC81" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD81" t="inlineStr"/>
@@ -12030,7 +12030,7 @@
       </c>
       <c r="AC82" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD82" t="inlineStr"/>
@@ -12175,7 +12175,7 @@
       </c>
       <c r="AC83" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD83" t="inlineStr"/>
@@ -12320,7 +12320,7 @@
       </c>
       <c r="AC84" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD84" t="inlineStr"/>
@@ -12465,7 +12465,7 @@
       </c>
       <c r="AC85" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD85" t="inlineStr"/>
@@ -12610,7 +12610,7 @@
       </c>
       <c r="AC86" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD86" t="inlineStr"/>
@@ -12752,7 +12752,7 @@
       </c>
       <c r="AC87" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD87" t="inlineStr"/>
@@ -13028,7 +13028,7 @@
       </c>
       <c r="AC89" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD89" t="inlineStr"/>
@@ -13304,7 +13304,7 @@
       </c>
       <c r="AC91" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD91" t="inlineStr"/>
@@ -13449,7 +13449,7 @@
       </c>
       <c r="AC92" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD92" t="inlineStr"/>
@@ -13594,7 +13594,7 @@
       </c>
       <c r="AC93" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD93" t="inlineStr"/>
@@ -13998,7 +13998,7 @@
       </c>
       <c r="AC96" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD96" t="inlineStr"/>
@@ -14143,7 +14143,7 @@
       </c>
       <c r="AC97" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD97" t="inlineStr"/>
@@ -14419,7 +14419,7 @@
       </c>
       <c r="AC99" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD99" t="inlineStr"/>
@@ -14564,7 +14564,7 @@
       </c>
       <c r="AC100" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD100" t="inlineStr"/>
@@ -14709,7 +14709,7 @@
       </c>
       <c r="AC101" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD101" t="inlineStr"/>
@@ -14854,7 +14854,7 @@
       </c>
       <c r="AC102" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD102" t="inlineStr"/>
@@ -15244,7 +15244,7 @@
       </c>
       <c r="AC105" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD105" t="inlineStr"/>
@@ -15389,7 +15389,7 @@
       </c>
       <c r="AC106" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD106" t="inlineStr"/>
@@ -15534,7 +15534,7 @@
       </c>
       <c r="AC107" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD107" t="inlineStr"/>
@@ -15679,7 +15679,7 @@
       </c>
       <c r="AC108" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD108" t="inlineStr"/>
@@ -15823,7 +15823,7 @@
       </c>
       <c r="AC109" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD109" t="inlineStr"/>
@@ -15968,7 +15968,7 @@
       </c>
       <c r="AC110" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD110" t="inlineStr"/>
@@ -16113,7 +16113,7 @@
       </c>
       <c r="AC111" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD111" t="inlineStr"/>
@@ -16258,7 +16258,7 @@
       </c>
       <c r="AC112" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD112" t="inlineStr"/>
@@ -16403,7 +16403,7 @@
       </c>
       <c r="AC113" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD113" t="inlineStr"/>
@@ -16548,7 +16548,7 @@
       </c>
       <c r="AC114" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD114" t="inlineStr"/>
@@ -16693,7 +16693,7 @@
       </c>
       <c r="AC115" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD115" t="inlineStr"/>
@@ -16838,7 +16838,7 @@
       </c>
       <c r="AC116" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD116" t="inlineStr"/>
@@ -16983,7 +16983,7 @@
       </c>
       <c r="AC117" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD117" t="inlineStr"/>
@@ -17128,7 +17128,7 @@
       </c>
       <c r="AC118" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD118" t="inlineStr"/>
@@ -17273,7 +17273,7 @@
       </c>
       <c r="AC119" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD119" t="inlineStr"/>
@@ -17418,7 +17418,7 @@
       </c>
       <c r="AC120" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD120" t="inlineStr"/>
@@ -17563,7 +17563,7 @@
       </c>
       <c r="AC121" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD121" t="inlineStr"/>
@@ -17708,7 +17708,7 @@
       </c>
       <c r="AC122" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD122" t="inlineStr"/>
@@ -17986,7 +17986,7 @@
       </c>
       <c r="AC124" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD124" t="inlineStr"/>
@@ -18670,7 +18670,7 @@
       </c>
       <c r="AC129" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD129" t="inlineStr"/>
@@ -18814,7 +18814,7 @@
       </c>
       <c r="AC130" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD130" t="inlineStr"/>
@@ -19229,7 +19229,7 @@
       </c>
       <c r="AC133" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD133" t="inlineStr"/>
@@ -19508,7 +19508,7 @@
       </c>
       <c r="AC135" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD135" t="inlineStr"/>
@@ -19653,7 +19653,7 @@
       </c>
       <c r="AC136" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD136" t="inlineStr"/>
@@ -20066,7 +20066,7 @@
       </c>
       <c r="AC139" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD139" t="inlineStr"/>
@@ -20613,7 +20613,7 @@
       </c>
       <c r="AC143" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD143" t="inlineStr"/>
@@ -21699,7 +21699,7 @@
       </c>
       <c r="AC151" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD151" t="inlineStr"/>
@@ -21842,7 +21842,7 @@
       </c>
       <c r="AC152" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD152" t="inlineStr"/>
@@ -22122,7 +22122,7 @@
       </c>
       <c r="AC154" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD154" t="inlineStr"/>
@@ -22267,7 +22267,7 @@
       </c>
       <c r="AC155" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD155" t="inlineStr"/>
@@ -22682,7 +22682,7 @@
       </c>
       <c r="AC158" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD158" t="inlineStr"/>
@@ -23097,7 +23097,7 @@
       </c>
       <c r="AC161" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD161" t="inlineStr"/>
@@ -23377,7 +23377,7 @@
       </c>
       <c r="AC163" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD163" t="inlineStr"/>
@@ -23650,7 +23650,7 @@
       </c>
       <c r="AC165" t="inlineStr">
         <is>
-          <t>2026-08-15 15:48:44</t>
+          <t>2026-08-15 16:02:04</t>
         </is>
       </c>
       <c r="AD165" t="inlineStr"/>

</xml_diff>